<commit_message>
refactor(elearning): modularize handlers, fix mapel grouping, fix sesi calculation, and add auto-select kelas on load
</commit_message>
<xml_diff>
--- a/public/templates/NILAI WARGA BELAJAR REKAP.xlsx
+++ b/public/templates/NILAI WARGA BELAJAR REKAP.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72F4F41-5883-45E5-BA40-557AB91A45BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C15584-420F-461D-90C9-8F4A137E13D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
   <si>
     <t>YAYASAN MENUJU MAKMUR</t>
   </si>
@@ -181,6 +181,9 @@
   <si>
     <t>NIP. ${nipWaliKelas}</t>
   </si>
+  <si>
+    <t>PKBM MENUJU MAKMUR</t>
+  </si>
 </sst>
 </file>
 
@@ -209,20 +212,6 @@
       <name val="Oceanic Drift"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="1"/>
-      <name val="Rockwell Extra Bold"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Cambria"/>
-      <family val="1"/>
-    </font>
-    <font>
       <i/>
       <sz val="10"/>
       <color theme="1"/>
@@ -454,6 +443,20 @@
       <color theme="1"/>
       <name val="Georgia"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="30"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -806,141 +809,138 @@
   </borders>
   <cellStyleXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="43" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="41" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="41" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="43" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="41" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="43" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="41" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="41" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="43" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="41" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1022,84 +1022,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>818027</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>45944</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>437027</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>327774</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="WordArt 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeArrowheads="1" noChangeShapeType="1" noTextEdit="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="2117909" y="236444"/>
-          <a:ext cx="5109883" cy="281830"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:extLst>
-          <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:effectLst/>
-            </a14:hiddenEffects>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="none" fromWordArt="1">
-          <a:prstTxWarp prst="textPlain">
-            <a:avLst>
-              <a:gd name="adj" fmla="val 50000"/>
-            </a:avLst>
-          </a:prstTxWarp>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:buNone/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="id-ID" sz="3600" b="1" kern="10" spc="0">
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:round/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a:ln>
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Hobo Std"/>
-            </a:rPr>
-            <a:t>PKBM MENUJU MAKMUR</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
@@ -1509,309 +1431,312 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="3" customWidth="1"/>
     <col min="4" max="4" width="27.28515625" style="1" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="13" style="6" customWidth="1"/>
-    <col min="9" max="10" width="12.7109375" style="6" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="13" style="4" customWidth="1"/>
+    <col min="9" max="10" width="12.7109375" style="4" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
     </row>
     <row r="2" spans="1:10" ht="27.75" customHeight="1">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
+      <c r="A2" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1" thickBot="1">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
     </row>
     <row r="7" spans="1:10" ht="7.5" customHeight="1" thickTop="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
     </row>
     <row r="8" spans="1:10" ht="7.5" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="33"/>
-      <c r="C13" s="16" t="s">
+      <c r="B13" s="32"/>
+      <c r="C13" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="5" t="s">
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="14"/>
+      <c r="C14" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="15"/>
-      <c r="I14" s="5"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="13"/>
+      <c r="I14" s="3"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="16"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:13" s="2" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F17" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23" t="s">
+      <c r="H17" s="33"/>
+      <c r="I17" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="J17" s="23"/>
+      <c r="J17" s="33"/>
     </row>
     <row r="18" spans="1:13" s="2" customFormat="1" ht="29.1" customHeight="1">
-      <c r="A18" s="34"/>
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="18" t="s">
+      <c r="A18" s="33"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H18" s="18" t="s">
+      <c r="H18" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="I18" s="18" t="s">
+      <c r="I18" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="J18" s="18" t="s">
+      <c r="J18" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:13" s="2" customFormat="1" ht="29.1" customHeight="1">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="J19" s="9" t="s">
+      <c r="J19" s="7" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1823,7 +1748,7 @@
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="1:13" ht="15" customHeight="1">
-      <c r="A23" s="8"/>
+      <c r="A23" s="6"/>
       <c r="B23" s="22" t="s">
         <v>14</v>
       </c>
@@ -1833,19 +1758,19 @@
       <c r="F23" s="22"/>
       <c r="G23" s="22"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
     </row>
     <row r="24" spans="1:13" ht="15" customHeight="1">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="8"/>
-      <c r="D24" s="12"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="10"/>
       <c r="E24" s="1" t="s">
         <v>36</v>
       </c>
@@ -1856,74 +1781,74 @@
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:13" ht="15" customHeight="1">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="17"/>
-      <c r="I25" s="24"/>
-      <c r="J25" s="24"/>
-      <c r="K25" s="24"/>
-      <c r="L25" s="24"/>
-      <c r="M25" s="24"/>
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="15"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
     </row>
     <row r="26" spans="1:13">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
     </row>
     <row r="27" spans="1:13" ht="15" customHeight="1">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="15"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
     </row>
     <row r="28" spans="1:13" ht="15" customHeight="1">
-      <c r="A28" s="8"/>
-      <c r="B28" s="21" t="s">
+      <c r="A28" s="6"/>
+      <c r="B28" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="21"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="21" t="s">
+      <c r="C28" s="19"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="I28" s="21" t="s">
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="I28" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
     </row>
     <row r="29" spans="1:13" ht="15" customHeight="1">
-      <c r="A29" s="8"/>
+      <c r="A29" s="6"/>
       <c r="B29" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C29" s="1"/>
-      <c r="D29" s="13"/>
+      <c r="D29" s="11"/>
       <c r="E29" s="1" t="s">
         <v>42</v>
       </c>

</xml_diff>